<commit_message>
classificação de estados por região de entrega
</commit_message>
<xml_diff>
--- a/docs/prazos-e-fretes.xlsx
+++ b/docs/prazos-e-fretes.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="Prazos e Fretes" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Faixas de Peso" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Estados por Regiao" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="124">
   <si>
     <t xml:space="preserve">Vitrinifarne — Tabela de Prazos e Fretes por Região</t>
   </si>
@@ -129,6 +130,270 @@
   </si>
   <si>
     <t xml:space="preserve">Fonte do exemplo: frete base econômico de Sudeste - capitais (R$ 19,90), célula F10 da aba Prazos e Fretes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classificação de estados e capitais por região de entrega</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Define em qual linha da aba Prazos e Fretes cada destino se enquadra. Capitais usam a faixa de capital; demais municípios usam a faixa de interior.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sigla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faixa de prazo aplicável</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rio Branco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amapa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Macapa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazonas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manaus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Para</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rondonia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porto Velho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roraima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boa Vista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tocantins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palmas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alagoas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maceio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nordeste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bahia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salvador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fortaleza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maranhao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sao Luis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paraiba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joao Pessoa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pernambuco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recife</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piaui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teresina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rio Grande do Norte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Natal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sergipe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aracaju</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distrito Federal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brasilia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goiania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mato Grosso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuiaba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mato Grosso do Sul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo Grande</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espirito Santo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vitoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sudeste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minas Gerais</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belo Horizonte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rio de Janeiro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RJ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sao Paulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Curitiba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rio Grande do Sul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porto Alegre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santa Catarina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Florianopolis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Municipios do interior do Nordeste usam a faixa Nordeste - interior. Municipios do interior do Sudeste usam a faixa Sudeste - interior.</t>
   </si>
 </sst>
 </file>
@@ -1014,4 +1279,521 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>